<commit_message>
Launch: close signups, pricing cleanup, signature, sitemap/robots
</commit_message>
<xml_diff>
--- a/src/i18n/i18n-strings.xlsx
+++ b/src/i18n/i18n-strings.xlsx
@@ -31592,12 +31592,12 @@
       </c>
       <c r="B1422" s="21" t="inlineStr">
         <is>
-          <t>Don't have an account?</t>
+          <t>New to UniqueApex?</t>
         </is>
       </c>
       <c r="C1422" s="22" t="inlineStr">
         <is>
-          <t>Pas encore de compte?</t>
+          <t>Nouveau sur UniqueApex?</t>
         </is>
       </c>
       <c r="D1422" s="22" t="n"/>
@@ -31614,12 +31614,12 @@
       </c>
       <c r="B1423" s="21" t="inlineStr">
         <is>
-          <t>Create one →</t>
+          <t>Join the waitlist →</t>
         </is>
       </c>
       <c r="C1423" s="22" t="inlineStr">
         <is>
-          <t>Créez-en un →</t>
+          <t>Rejoignez la liste d'attente →</t>
         </is>
       </c>
       <c r="D1423" s="22" t="n"/>
@@ -62447,12 +62447,12 @@
       </c>
       <c r="B2829" s="21" t="inlineStr">
         <is>
-          <t>create an account</t>
+          <t>join the waitlist</t>
         </is>
       </c>
       <c r="C2829" s="22" t="inlineStr">
         <is>
-          <t>créer un compte</t>
+          <t>rejoindre la liste d'attente</t>
         </is>
       </c>
       <c r="D2829" s="22" t="n"/>
@@ -64455,7 +64455,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="15">
       <c r="A3" s="23" t="inlineStr">
         <is>

</xml_diff>